<commit_message>
Count a factor's first published year as a full stock change.
Late-starting SGS series (redesconto, derivativos, emergency lines)
were dropping out of the 2020 variation table because the prior year
was empty. Treat that debut as a change from zero.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/fatores_base_monetaria_tabelas_1995_2026.xlsx
+++ b/output/fatores_base_monetaria_tabelas_1995_2026.xlsx
@@ -860,7 +860,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0,0</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1,7</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>+16,0</t>
+          <t>+14,3</t>
         </is>
       </c>
     </row>
@@ -2010,12 +2010,12 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+27,8</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>+148,7</t>
+          <t>+120,9</t>
         </is>
       </c>
     </row>

</xml_diff>